<commit_message>
Standardize every source and separate raw data from plot inputs
</commit_message>
<xml_diff>
--- a/standardized/MA_42D_standardized.xlsx
+++ b/standardized/MA_42D_standardized.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'validation_check'!$A$1:$E$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'issues_if_any'!$A$1:$H$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'raw_observations'!$A$1:$I$701</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'normalization_notes'!$A$1:$B$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'normalization_notes'!$A$1:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,12 +513,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -530,16 +530,16 @@
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -555,12 +555,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -614,16 +614,16 @@
         <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -639,12 +639,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -656,16 +656,16 @@
         <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -681,12 +681,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -698,16 +698,16 @@
         <v>5</v>
       </c>
       <c r="G6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" t="n">
         <v>1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.2</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -723,12 +723,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -765,12 +765,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -782,16 +782,16 @@
         <v>5</v>
       </c>
       <c r="G8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -807,12 +807,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -823,11 +823,17 @@
       <c r="F9" t="n">
         <v>5</v>
       </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -843,12 +849,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -859,17 +865,11 @@
       <c r="F10" t="n">
         <v>5</v>
       </c>
-      <c r="G10" t="n">
-        <v>3</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.6</v>
-      </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -927,7 +927,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -944,16 +944,16 @@
         <v>5</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -969,7 +969,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1028,16 +1028,16 @@
         <v>5</v>
       </c>
       <c r="G14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" t="n">
         <v>1</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.2</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1090,22 +1090,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1132,32 +1132,38 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>5</v>
       </c>
+      <c r="G17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -1168,12 +1174,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1183,7 +1189,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1210,22 +1216,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1252,38 +1258,38 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>5</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -1294,38 +1300,38 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>5</v>
       </c>
       <c r="G21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -1336,22 +1342,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1378,38 +1384,38 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>5</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
@@ -1420,38 +1426,38 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F24" t="n">
         <v>5</v>
       </c>
       <c r="G24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -1462,7 +1468,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1477,7 +1483,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1504,12 +1510,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1519,23 +1525,23 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H26" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -1546,12 +1552,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1561,23 +1567,23 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>5</v>
       </c>
       <c r="G27" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -1588,12 +1594,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1603,23 +1609,23 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>5</v>
       </c>
       <c r="G28" t="n">
+        <v>5</v>
+      </c>
+      <c r="H28" t="n">
         <v>1</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0.2</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -1630,7 +1636,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1645,23 +1651,23 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>5</v>
       </c>
       <c r="G29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H29" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -1677,33 +1683,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>5</v>
       </c>
-      <c r="G30" t="n">
-        <v>5</v>
-      </c>
-      <c r="H30" t="n">
+      <c r="I30" t="n">
         <v>1</v>
       </c>
-      <c r="I30" t="n">
-        <v>0</v>
-      </c>
       <c r="J30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
@@ -1719,33 +1719,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>5</v>
       </c>
-      <c r="G31" t="n">
-        <v>2</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0.4</v>
-      </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -1761,7 +1755,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1771,23 +1765,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F32" t="n">
         <v>5</v>
       </c>
-      <c r="G32" t="n">
-        <v>5</v>
-      </c>
-      <c r="H32" t="n">
+      <c r="I32" t="n">
         <v>1</v>
       </c>
-      <c r="I32" t="n">
-        <v>0</v>
-      </c>
       <c r="J32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -1803,33 +1791,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F33" t="n">
         <v>5</v>
       </c>
-      <c r="G33" t="n">
-        <v>5</v>
-      </c>
-      <c r="H33" t="n">
+      <c r="I33" t="n">
         <v>1</v>
       </c>
-      <c r="I33" t="n">
+      <c r="J33" t="n">
         <v>0</v>
-      </c>
-      <c r="J33" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="34">
@@ -1845,17 +1827,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -1887,33 +1869,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F35" t="n">
         <v>5</v>
       </c>
-      <c r="G35" t="n">
-        <v>5</v>
-      </c>
-      <c r="H35" t="n">
+      <c r="I35" t="n">
         <v>1</v>
       </c>
-      <c r="I35" t="n">
+      <c r="J35" t="n">
         <v>0</v>
-      </c>
-      <c r="J35" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="36">
@@ -1929,17 +1905,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -1971,33 +1947,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F37" t="n">
         <v>5</v>
       </c>
-      <c r="G37" t="n">
-        <v>3</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.6</v>
-      </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38">
@@ -2013,33 +1983,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F38" t="n">
         <v>5</v>
       </c>
-      <c r="G38" t="n">
-        <v>5</v>
-      </c>
-      <c r="H38" t="n">
+      <c r="I38" t="n">
         <v>1</v>
       </c>
-      <c r="I38" t="n">
-        <v>0</v>
-      </c>
       <c r="J38" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -2065,7 +2029,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2097,7 +2061,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2107,23 +2071,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F40" t="n">
         <v>5</v>
       </c>
-      <c r="G40" t="n">
-        <v>5</v>
-      </c>
-      <c r="H40" t="n">
+      <c r="I40" t="n">
         <v>1</v>
       </c>
-      <c r="I40" t="n">
-        <v>0</v>
-      </c>
       <c r="J40" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -2139,7 +2097,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2149,7 +2107,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -2181,7 +2139,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2191,23 +2149,23 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F42" t="n">
         <v>5</v>
       </c>
       <c r="G42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H42" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
@@ -2233,23 +2191,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F43" t="n">
         <v>5</v>
       </c>
-      <c r="G43" t="n">
-        <v>5</v>
-      </c>
-      <c r="H43" t="n">
+      <c r="I43" t="n">
         <v>1</v>
       </c>
-      <c r="I43" t="n">
-        <v>0</v>
-      </c>
       <c r="J43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44">
@@ -2260,38 +2212,32 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>5</v>
       </c>
-      <c r="G44" t="n">
-        <v>5</v>
-      </c>
-      <c r="H44" t="n">
+      <c r="I44" t="n">
         <v>1</v>
       </c>
-      <c r="I44" t="n">
-        <v>0</v>
-      </c>
       <c r="J44" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
@@ -2302,38 +2248,32 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F45" t="n">
         <v>5</v>
       </c>
-      <c r="G45" t="n">
-        <v>4</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0.8</v>
-      </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="46">
@@ -2344,12 +2284,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2359,23 +2299,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>5</v>
       </c>
-      <c r="G46" t="n">
-        <v>4</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0.8</v>
-      </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J46" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -2386,38 +2320,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>5</v>
       </c>
-      <c r="G47" t="n">
-        <v>4</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0.8</v>
-      </c>
       <c r="I47" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" t="n">
         <v>0</v>
-      </c>
-      <c r="J47" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="48">
@@ -2428,22 +2356,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -2470,38 +2398,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>5</v>
       </c>
-      <c r="G49" t="n">
-        <v>5</v>
-      </c>
-      <c r="H49" t="n">
+      <c r="I49" t="n">
         <v>1</v>
       </c>
-      <c r="I49" t="n">
-        <v>0</v>
-      </c>
       <c r="J49" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -2512,22 +2434,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -2554,38 +2476,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F51" t="n">
         <v>5</v>
       </c>
-      <c r="G51" t="n">
-        <v>3</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0.6</v>
-      </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -2596,38 +2512,38 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F52" t="n">
         <v>5</v>
       </c>
       <c r="G52" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H52" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -2638,7 +2554,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2653,7 +2569,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2680,12 +2596,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2695,23 +2611,17 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F54" t="n">
         <v>5</v>
       </c>
-      <c r="G54" t="n">
-        <v>4</v>
-      </c>
-      <c r="H54" t="n">
-        <v>0.8</v>
-      </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J54" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
@@ -2722,12 +2632,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2737,7 +2647,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -2764,12 +2674,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2779,23 +2689,23 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F56" t="n">
         <v>5</v>
       </c>
       <c r="G56" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H56" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="I56" t="n">
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="57">
@@ -2806,7 +2716,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Gut</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2821,23 +2731,17 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F57" t="n">
         <v>5</v>
       </c>
-      <c r="G57" t="n">
-        <v>5</v>
-      </c>
-      <c r="H57" t="n">
+      <c r="I57" t="n">
+        <v>2</v>
+      </c>
+      <c r="J57" t="n">
         <v>1</v>
-      </c>
-      <c r="I57" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="58">
@@ -2853,33 +2757,33 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F58" t="n">
         <v>5</v>
       </c>
       <c r="G58" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H58" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="59">
@@ -2895,30 +2799,24 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F59" t="n">
         <v>5</v>
       </c>
-      <c r="G59" t="n">
-        <v>4</v>
-      </c>
-      <c r="H59" t="n">
-        <v>0.8</v>
-      </c>
       <c r="I59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J59" t="n">
         <v>4</v>
@@ -2937,7 +2835,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2947,23 +2845,23 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F60" t="n">
         <v>5</v>
       </c>
       <c r="G60" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H60" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I60" t="n">
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
@@ -2979,27 +2877,33 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F61" t="n">
         <v>5</v>
       </c>
+      <c r="G61" t="n">
+        <v>2</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.4</v>
+      </c>
       <c r="I61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
@@ -3015,27 +2919,33 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F62" t="n">
         <v>5</v>
       </c>
+      <c r="G62" t="n">
+        <v>3</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.6</v>
+      </c>
       <c r="I62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63">
@@ -3051,24 +2961,30 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F63" t="n">
         <v>5</v>
       </c>
+      <c r="G63" t="n">
+        <v>4</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.8</v>
+      </c>
       <c r="I63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J63" t="n">
         <v>4</v>
@@ -3087,27 +3003,33 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F64" t="n">
         <v>5</v>
       </c>
+      <c r="G64" t="n">
+        <v>5</v>
+      </c>
+      <c r="H64" t="n">
+        <v>1</v>
+      </c>
       <c r="I64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65">
@@ -3123,27 +3045,33 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F65" t="n">
         <v>5</v>
       </c>
+      <c r="G65" t="n">
+        <v>4</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0.8</v>
+      </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66">
@@ -3159,27 +3087,33 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F66" t="n">
         <v>5</v>
       </c>
+      <c r="G66" t="n">
+        <v>3</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0.6</v>
+      </c>
       <c r="I66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67">
@@ -3205,7 +3139,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -3237,7 +3171,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3247,23 +3181,23 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F68" t="n">
         <v>5</v>
       </c>
       <c r="G68" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I68" t="n">
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -3279,7 +3213,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3289,7 +3223,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -3299,7 +3233,7 @@
         <v>1</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="70">
@@ -3315,7 +3249,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3325,17 +3259,23 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F70" t="n">
         <v>5</v>
       </c>
+      <c r="G70" t="n">
+        <v>5</v>
+      </c>
+      <c r="H70" t="n">
+        <v>1</v>
+      </c>
       <c r="I70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
@@ -3361,17 +3301,23 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="F71" t="n">
         <v>5</v>
       </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
       <c r="I71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -3387,17 +3333,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -3429,33 +3375,33 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F73" t="n">
         <v>5</v>
       </c>
       <c r="G73" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H73" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I73" t="n">
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="74">
@@ -3471,7 +3417,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3481,23 +3427,23 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F74" t="n">
         <v>5</v>
       </c>
       <c r="G74" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H74" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="I74" t="n">
         <v>0</v>
       </c>
       <c r="J74" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75">
@@ -3513,33 +3459,33 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F75" t="n">
         <v>5</v>
       </c>
       <c r="G75" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I75" t="n">
         <v>0</v>
       </c>
       <c r="J75" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -3555,33 +3501,33 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F76" t="n">
         <v>5</v>
       </c>
       <c r="G76" t="n">
+        <v>5</v>
+      </c>
+      <c r="H76" t="n">
         <v>1</v>
-      </c>
-      <c r="H76" t="n">
-        <v>0.2</v>
       </c>
       <c r="I76" t="n">
         <v>0</v>
       </c>
       <c r="J76" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="77">
@@ -3597,33 +3543,33 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F77" t="n">
         <v>5</v>
       </c>
       <c r="G77" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H77" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I77" t="n">
         <v>0</v>
       </c>
       <c r="J77" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78">
@@ -3639,33 +3585,33 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F78" t="n">
         <v>5</v>
       </c>
       <c r="G78" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H78" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I78" t="n">
         <v>0</v>
       </c>
       <c r="J78" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="79">
@@ -3681,33 +3627,33 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F79" t="n">
         <v>5</v>
       </c>
       <c r="G79" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H79" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="I79" t="n">
         <v>0</v>
       </c>
       <c r="J79" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80">
@@ -3723,33 +3669,33 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F80" t="n">
         <v>5</v>
       </c>
       <c r="G80" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H80" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="I80" t="n">
         <v>0</v>
       </c>
       <c r="J80" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -3775,7 +3721,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -3807,7 +3753,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3817,23 +3763,23 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F82" t="n">
         <v>5</v>
       </c>
       <c r="G82" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H82" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I82" t="n">
         <v>0</v>
       </c>
       <c r="J82" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -3849,7 +3795,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3859,23 +3805,17 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F83" t="n">
         <v>5</v>
       </c>
-      <c r="G83" t="n">
-        <v>3</v>
-      </c>
-      <c r="H83" t="n">
-        <v>0.6</v>
-      </c>
       <c r="I83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J83" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84">
@@ -3891,7 +3831,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3901,23 +3841,23 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F84" t="n">
         <v>5</v>
       </c>
       <c r="G84" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H84" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="I84" t="n">
         <v>0</v>
       </c>
       <c r="J84" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="85">
@@ -3943,7 +3883,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -3970,38 +3910,38 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F86" t="n">
         <v>5</v>
       </c>
       <c r="G86" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H86" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="I86" t="n">
         <v>0</v>
       </c>
       <c r="J86" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="87">
@@ -4012,22 +3952,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -4054,12 +3994,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4069,23 +4009,23 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F88" t="n">
         <v>5</v>
       </c>
       <c r="G88" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H88" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I88" t="n">
         <v>0</v>
       </c>
       <c r="J88" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89">
@@ -4096,32 +4036,38 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F89" t="n">
         <v>5</v>
       </c>
+      <c r="G89" t="n">
+        <v>5</v>
+      </c>
+      <c r="H89" t="n">
+        <v>1</v>
+      </c>
       <c r="I89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="90">
@@ -4132,32 +4078,38 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F90" t="n">
         <v>5</v>
       </c>
+      <c r="G90" t="n">
+        <v>4</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0.8</v>
+      </c>
       <c r="I90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J90" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91">
@@ -4168,29 +4120,35 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F91" t="n">
         <v>5</v>
       </c>
+      <c r="G91" t="n">
+        <v>3</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0.6</v>
+      </c>
       <c r="I91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J91" t="n">
         <v>3</v>
@@ -4204,32 +4162,38 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F92" t="n">
         <v>5</v>
       </c>
+      <c r="G92" t="n">
+        <v>5</v>
+      </c>
+      <c r="H92" t="n">
+        <v>1</v>
+      </c>
       <c r="I92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J92" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="93">
@@ -4240,38 +4204,38 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F93" t="n">
         <v>5</v>
       </c>
       <c r="G93" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H93" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="I93" t="n">
         <v>0</v>
       </c>
       <c r="J93" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94">
@@ -4282,32 +4246,38 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F94" t="n">
         <v>5</v>
       </c>
+      <c r="G94" t="n">
+        <v>3</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0.6</v>
+      </c>
       <c r="I94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J94" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95">
@@ -4318,7 +4288,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4333,7 +4303,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -4360,12 +4330,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -4375,23 +4345,23 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F96" t="n">
         <v>5</v>
       </c>
       <c r="G96" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H96" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="I96" t="n">
         <v>0</v>
       </c>
       <c r="J96" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="97">
@@ -4402,12 +4372,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4417,17 +4387,23 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F97" t="n">
         <v>5</v>
       </c>
+      <c r="G97" t="n">
+        <v>4</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0.8</v>
+      </c>
       <c r="I97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J97" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="98">
@@ -4438,12 +4414,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4453,17 +4429,23 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F98" t="n">
         <v>5</v>
       </c>
+      <c r="G98" t="n">
+        <v>4</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0.8</v>
+      </c>
       <c r="I98" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J98" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="99">
@@ -4474,7 +4456,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4489,17 +4471,23 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="F99" t="n">
         <v>5</v>
       </c>
+      <c r="G99" t="n">
+        <v>5</v>
+      </c>
+      <c r="H99" t="n">
+        <v>1</v>
+      </c>
       <c r="I99" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J99" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="100">
@@ -4515,33 +4503,33 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F100" t="n">
         <v>5</v>
       </c>
       <c r="G100" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H100" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I100" t="n">
         <v>0</v>
       </c>
       <c r="J100" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="101">
@@ -4557,33 +4545,33 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F101" t="n">
         <v>5</v>
       </c>
       <c r="G101" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H101" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I101" t="n">
         <v>0</v>
       </c>
       <c r="J101" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="102">
@@ -4599,7 +4587,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -4609,23 +4597,23 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F102" t="n">
         <v>5</v>
       </c>
       <c r="G102" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H102" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I102" t="n">
         <v>0</v>
       </c>
       <c r="J102" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="103">
@@ -4641,27 +4629,33 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F103" t="n">
         <v>5</v>
       </c>
+      <c r="G103" t="n">
+        <v>1</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0.2</v>
+      </c>
       <c r="I103" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -4677,33 +4671,33 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F104" t="n">
         <v>5</v>
       </c>
       <c r="G104" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I104" t="n">
         <v>0</v>
       </c>
       <c r="J104" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="105">
@@ -4719,27 +4713,33 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F105" t="n">
         <v>5</v>
       </c>
+      <c r="G105" t="n">
+        <v>3</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0.6</v>
+      </c>
       <c r="I105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J105" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="106">
@@ -4755,17 +4755,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -4797,33 +4797,33 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F107" t="n">
         <v>5</v>
       </c>
       <c r="G107" t="n">
+        <v>5</v>
+      </c>
+      <c r="H107" t="n">
         <v>1</v>
-      </c>
-      <c r="H107" t="n">
-        <v>0.2</v>
       </c>
       <c r="I107" t="n">
         <v>0</v>
       </c>
       <c r="J107" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="108">
@@ -4839,33 +4839,33 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F108" t="n">
         <v>5</v>
       </c>
       <c r="G108" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H108" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I108" t="n">
         <v>0</v>
       </c>
       <c r="J108" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F109" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -4933,14 +4933,20 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F110" t="n">
         <v>5</v>
       </c>
+      <c r="G110" t="n">
+        <v>3</v>
+      </c>
+      <c r="H110" t="n">
+        <v>0.6</v>
+      </c>
       <c r="I110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J110" t="n">
         <v>3</v>
@@ -4959,7 +4965,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -4969,23 +4975,23 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F111" t="n">
         <v>5</v>
       </c>
       <c r="G111" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H111" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="I111" t="n">
         <v>0</v>
       </c>
       <c r="J111" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="112">
@@ -5001,7 +5007,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -5011,23 +5017,23 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F112" t="n">
         <v>5</v>
       </c>
       <c r="G112" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I112" t="n">
         <v>0</v>
       </c>
       <c r="J112" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113">
@@ -5053,23 +5059,23 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="F113" t="n">
         <v>5</v>
       </c>
       <c r="G113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H113" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I113" t="n">
         <v>0</v>
       </c>
       <c r="J113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114">
@@ -5080,38 +5086,32 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F114" t="n">
         <v>5</v>
       </c>
-      <c r="G114" t="n">
-        <v>5</v>
-      </c>
-      <c r="H114" t="n">
+      <c r="I114" t="n">
         <v>1</v>
       </c>
-      <c r="I114" t="n">
-        <v>0</v>
-      </c>
       <c r="J114" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="115">
@@ -5122,32 +5122,38 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F115" t="n">
         <v>5</v>
       </c>
+      <c r="G115" t="n">
+        <v>5</v>
+      </c>
+      <c r="H115" t="n">
+        <v>1</v>
+      </c>
       <c r="I115" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J115" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="116">
@@ -5158,12 +5164,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -5173,23 +5179,23 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F116" t="n">
         <v>5</v>
       </c>
       <c r="G116" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H116" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I116" t="n">
         <v>0</v>
       </c>
       <c r="J116" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -5200,38 +5206,38 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F117" t="n">
         <v>5</v>
       </c>
       <c r="G117" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H117" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="I117" t="n">
         <v>0</v>
       </c>
       <c r="J117" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -5242,38 +5248,32 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F118" t="n">
         <v>5</v>
       </c>
-      <c r="G118" t="n">
-        <v>2</v>
-      </c>
-      <c r="H118" t="n">
-        <v>0.4</v>
-      </c>
       <c r="I118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J118" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="119">
@@ -5284,38 +5284,38 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F119" t="n">
         <v>5</v>
       </c>
       <c r="G119" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H119" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="I119" t="n">
         <v>0</v>
       </c>
       <c r="J119" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120">
@@ -5326,32 +5326,38 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F120" t="n">
         <v>5</v>
       </c>
+      <c r="G120" t="n">
+        <v>5</v>
+      </c>
+      <c r="H120" t="n">
+        <v>1</v>
+      </c>
       <c r="I120" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J120" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="121">
@@ -5362,38 +5368,32 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F121" t="n">
         <v>5</v>
       </c>
-      <c r="G121" t="n">
-        <v>3</v>
-      </c>
-      <c r="H121" t="n">
-        <v>0.6</v>
-      </c>
       <c r="I121" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J121" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122">
@@ -5404,38 +5404,38 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F122" t="n">
         <v>5</v>
       </c>
       <c r="G122" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H122" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="I122" t="n">
         <v>0</v>
       </c>
       <c r="J122" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5461,7 +5461,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -5488,12 +5488,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -5503,23 +5503,23 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F124" t="n">
         <v>5</v>
       </c>
       <c r="G124" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H124" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="I124" t="n">
         <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125">
@@ -5530,12 +5530,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -5545,23 +5545,23 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F125" t="n">
         <v>5</v>
       </c>
       <c r="G125" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H125" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I125" t="n">
         <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="126">
@@ -5572,12 +5572,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -5587,23 +5587,23 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F126" t="n">
         <v>5</v>
       </c>
       <c r="G126" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I126" t="n">
         <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="127">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Gut</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5629,23 +5629,23 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="F127" t="n">
         <v>5</v>
       </c>
       <c r="G127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H127" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I127" t="n">
         <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -5661,12 +5661,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Pseudoalteromonas piratica</t>
+          <t>Bacillus altitudinis</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Firmicutes</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -5678,16 +5678,16 @@
         <v>5</v>
       </c>
       <c r="G128" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H128" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I128" t="n">
         <v>0</v>
       </c>
       <c r="J128" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="129">
@@ -5703,12 +5703,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Vibrio jasicida</t>
+          <t>Demequina globuliformis</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Actinobacteria</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Vibrio owensii</t>
+          <t>Litorilituus sediminis</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -5761,11 +5761,17 @@
       <c r="F130" t="n">
         <v>5</v>
       </c>
+      <c r="G130" t="n">
+        <v>3</v>
+      </c>
+      <c r="H130" t="n">
+        <v>0.6</v>
+      </c>
       <c r="I130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="131">
@@ -5781,12 +5787,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Ruegeria profundi</t>
+          <t>Mesoflavibacter zeaxanthinifaciens</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -5798,16 +5804,16 @@
         <v>5</v>
       </c>
       <c r="G131" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H131" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I131" t="n">
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
@@ -5823,12 +5829,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Mesoflavibacter zeaxanthinifaciens</t>
+          <t>Paracoccus homiensis</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -5840,16 +5846,16 @@
         <v>5</v>
       </c>
       <c r="G132" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H132" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="I132" t="n">
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="133">
@@ -5865,12 +5871,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Bacillus altitudinis</t>
+          <t>Photobacterium damselae</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Firmicutes</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -5882,16 +5888,16 @@
         <v>5</v>
       </c>
       <c r="G133" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H133" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I133" t="n">
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="134">
@@ -5907,12 +5913,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Demequina globuliformis</t>
+          <t>Pseudoalteromonas piratica</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Actinobacteria</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -5949,12 +5955,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Tenacibaculum discolor</t>
+          <t>Ruegeria profundi</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Bacteroidota</t>
+          <t>Proteobacteria</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5966,16 +5972,16 @@
         <v>5</v>
       </c>
       <c r="G135" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H135" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="I135" t="n">
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="136">
@@ -5991,12 +5997,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Litorilituus sediminis</t>
+          <t>Tenacibaculum discolor</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Proteobacteria</t>
+          <t>Bacteroidota</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -6075,7 +6081,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Paracoccus homiensis</t>
+          <t>Vibrio brasiliensis</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -6092,16 +6098,16 @@
         <v>5</v>
       </c>
       <c r="G138" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H138" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="I138" t="n">
         <v>0</v>
       </c>
       <c r="J138" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="139">
@@ -6117,7 +6123,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Photobacterium damselae</t>
+          <t>Vibrio jasicida</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -6159,7 +6165,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Vibrio brasiliensis</t>
+          <t>Vibrio owensii</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -6175,17 +6181,11 @@
       <c r="F140" t="n">
         <v>5</v>
       </c>
-      <c r="G140" t="n">
-        <v>2</v>
-      </c>
-      <c r="H140" t="n">
-        <v>0.4</v>
-      </c>
       <c r="I140" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J140" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="141">
@@ -36377,7 +36377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -36411,151 +36411,175 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sha256</t>
+          <t>rawPath</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f1ca1afdd19568bd1385e7399f5d932845b1ef083ea64bf1af4673d6031d389b</t>
+          <t>raw/MA_42D.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>method</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DOC42</t>
+          <t>individual_shrimp_presence</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>blankPolicy</t>
+          <t>sha256</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>f1ca1afdd19568bd1385e7399f5d932845b1ef083ea64bf1af4673d6031d389b</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rawSamples</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>50</v>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DOC42</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rawMeasurements</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>700</v>
+          <t>blankPolicy</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>missingMeasurements</t>
+          <t>rawSamples</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>28</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>summaryRows</t>
+          <t>rawMeasurements</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>140</v>
+        <v>700</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>incompleteSummaries</t>
+          <t>missingMeasurements</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Positive rule</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Measurement &gt; 0; dilution does not change presence/absence.</t>
-        </is>
+          <t>summaryRows</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>140</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Blank rule</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Unknown, not zero. Any blank makes the cohort/taxon percentage unknown.</t>
-        </is>
+          <t>incompleteSummaries</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Organ mapping</t>
+          <t>Positive rule</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>G -&gt; Gut; HP -&gt; HP</t>
+          <t>Measurement &gt; 0; dilution does not change presence/absence.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Identifiers</t>
+          <t>Blank rule</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Treatment and shrimp identifiers resolved only through actual merged ranges.</t>
+          <t>Unknown, not zero. Any blank makes the cohort/taxon percentage unknown.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Organ mapping</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>G -&gt; Gut; HP -&gt; HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Identifiers</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Treatment and shrimp identifiers resolved only through actual merged ranges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Time label</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>DOC42 from the user-specified sampling source MA_42D.xlsx.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B15"/>
+  <autoFilter ref="A1:B17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>